<commit_message>
fixed hover on yearly avg temp graph added code to produce windrose for LISICOS directly in markdown vs displaying png.
</commit_message>
<xml_diff>
--- a/data/YearlyAvgTemp_pivot2.xlsx
+++ b/data/YearlyAvgTemp_pivot2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\R\Projects\2025 Hypoxia Summary\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\R\Projects\2025 Hypoxia Summary\2025_Hypoxia_Season_Summary\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FF71D3A-C3B9-427C-9C9E-C5DD2FAB7157}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBAEB154-AD85-4EA1-BC37-2F0BF66B9044}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{8D51FA5F-2FE8-455D-8B35-A72003373017}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{8D51FA5F-2FE8-455D-8B35-A72003373017}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -754,7 +754,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{086B91A9-BCA8-4DF2-8B79-0210994E455D}">
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.6640625" style="1" bestFit="1" customWidth="1"/>
@@ -775,396 +775,403 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
-        <v>1991</v>
-      </c>
-      <c r="B2" s="3">
-        <v>14.551219642857145</v>
-      </c>
-      <c r="C2" s="2">
-        <v>13.267019642857147</v>
+        <v>1990</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
-        <v>1992</v>
-      </c>
-      <c r="B3" s="4">
-        <v>12.207588059701498</v>
+        <v>1991</v>
+      </c>
+      <c r="B3" s="3">
+        <v>14.551219642857145</v>
       </c>
       <c r="C3" s="2">
-        <v>11.084627536231885</v>
+        <v>13.267019642857147</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
-        <v>1993</v>
+        <v>1992</v>
       </c>
       <c r="B4" s="4">
-        <v>15.273027450980393</v>
+        <v>12.207588059701498</v>
       </c>
       <c r="C4" s="2">
-        <v>11.258387500000001</v>
+        <v>11.084627536231885</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
-        <v>1994</v>
+        <v>1993</v>
       </c>
       <c r="B5" s="4">
-        <v>18.482944557823128</v>
+        <v>15.273027450980393</v>
       </c>
       <c r="C5" s="2">
-        <v>10.109010112359549</v>
+        <v>11.258387500000001</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
-        <v>1995</v>
+        <v>1994</v>
       </c>
       <c r="B6" s="4">
-        <v>11.141750000000004</v>
+        <v>18.482944557823128</v>
       </c>
       <c r="C6" s="2">
-        <v>12.347900425531918</v>
+        <v>10.109010112359549</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
-        <v>1996</v>
+        <v>1995</v>
       </c>
       <c r="B7" s="4">
-        <v>16.653554193548384</v>
+        <v>11.141750000000004</v>
       </c>
       <c r="C7" s="2">
-        <v>11.966351612903221</v>
+        <v>12.347900425531918</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
-        <v>1997</v>
+        <v>1996</v>
       </c>
       <c r="B8" s="4">
-        <v>16.192166785714303</v>
+        <v>16.653554193548384</v>
       </c>
       <c r="C8" s="2">
-        <v>12.117467142857132</v>
+        <v>11.966351612903221</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
-        <v>1998</v>
+        <v>1997</v>
       </c>
       <c r="B9" s="4">
-        <v>17.803113086419746</v>
+        <v>16.192166785714303</v>
       </c>
       <c r="C9" s="2">
-        <v>12.941916194331982</v>
+        <v>12.117467142857132</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
-        <v>1999</v>
+        <v>1998</v>
       </c>
       <c r="B10" s="4">
-        <v>17.134333080808073</v>
+        <v>17.803113086419746</v>
       </c>
       <c r="C10" s="2">
-        <v>12.311642187500002</v>
+        <v>12.941916194331982</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
-        <v>2000</v>
+        <v>1999</v>
       </c>
       <c r="B11" s="4">
-        <v>16.633897169811313</v>
+        <v>17.134333080808073</v>
       </c>
       <c r="C11" s="2">
-        <v>12.032005490196077</v>
+        <v>12.311642187500002</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
-        <v>2001</v>
+        <v>2000</v>
       </c>
       <c r="B12" s="4">
-        <v>17.681043410852713</v>
+        <v>16.633897169811313</v>
       </c>
       <c r="C12" s="2">
-        <v>12.926708870967744</v>
+        <v>12.032005490196077</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
-        <v>2002</v>
+        <v>2001</v>
       </c>
       <c r="B13" s="4">
-        <v>14.909986131386866</v>
+        <v>17.681043410852713</v>
       </c>
       <c r="C13" s="2">
-        <v>12.440276446280995</v>
+        <v>12.926708870967744</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
-        <v>2003</v>
+        <v>2002</v>
       </c>
       <c r="B14" s="4">
-        <v>15.669723939393942</v>
+        <v>14.909986131386866</v>
       </c>
       <c r="C14" s="2">
-        <v>11.341413122171941</v>
+        <v>12.440276446280995</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
-        <v>2004</v>
+        <v>2003</v>
       </c>
       <c r="B15" s="4">
-        <v>17.035140955631395</v>
+        <v>15.669723939393942</v>
       </c>
       <c r="C15" s="2">
-        <v>12.645331018518515</v>
+        <v>11.341413122171941</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
-        <v>2005</v>
+        <v>2004</v>
       </c>
       <c r="B16" s="4">
-        <v>17.502046979865781</v>
+        <v>17.035140955631395</v>
       </c>
       <c r="C16" s="2">
-        <v>12.443033596837953</v>
+        <v>12.645331018518515</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
-        <v>2006</v>
+        <v>2005</v>
       </c>
       <c r="B17" s="4">
-        <v>18.666583448275865</v>
+        <v>17.502046979865781</v>
       </c>
       <c r="C17" s="2">
-        <v>14.990842543859658</v>
+        <v>12.443033596837953</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
-        <v>2007</v>
+        <v>2006</v>
       </c>
       <c r="B18" s="4">
-        <v>16.781344444444443</v>
+        <v>18.666583448275865</v>
       </c>
       <c r="C18" s="2">
-        <v>12.764724031007752</v>
+        <v>14.990842543859658</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
-        <v>2008</v>
+        <v>2007</v>
       </c>
       <c r="B19" s="4">
-        <v>16.463443296089384</v>
+        <v>16.781344444444443</v>
       </c>
       <c r="C19" s="2">
-        <v>12.130273200000001</v>
+        <v>12.764724031007752</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
-        <v>2009</v>
+        <v>2008</v>
       </c>
       <c r="B20" s="4">
-        <v>14.864309900990094</v>
+        <v>16.463443296089384</v>
       </c>
       <c r="C20" s="2">
-        <v>11.574757199999999</v>
+        <v>12.130273200000001</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
-        <v>2010</v>
+        <v>2009</v>
       </c>
       <c r="B21" s="4">
-        <v>16.380146263345218</v>
+        <v>14.864309900990094</v>
       </c>
       <c r="C21" s="2">
-        <v>12.756010204081635</v>
+        <v>11.574757199999999</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
-        <v>2011</v>
+        <v>2010</v>
       </c>
       <c r="B22" s="4">
-        <v>16.757059878419451</v>
+        <v>16.380146263345218</v>
       </c>
       <c r="C22" s="2">
-        <v>11.92756696832579</v>
+        <v>12.756010204081635</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="1">
-        <v>2012</v>
+        <v>2011</v>
       </c>
       <c r="B23" s="4">
-        <v>17.683542821158689</v>
+        <v>16.757059878419451</v>
       </c>
       <c r="C23" s="2">
-        <v>13.661042471042471</v>
+        <v>11.92756696832579</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" s="1">
-        <v>2013</v>
+        <v>2012</v>
       </c>
       <c r="B24" s="4">
-        <v>17.140527525252523</v>
+        <v>17.683542821158689</v>
       </c>
       <c r="C24" s="2">
-        <v>12.939243461538458</v>
+        <v>13.661042471042471</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
-        <v>2014</v>
+        <v>2013</v>
       </c>
       <c r="B25" s="4">
-        <v>16.304540920716121</v>
+        <v>17.140527525252523</v>
       </c>
       <c r="C25" s="2">
-        <v>11.953458687258692</v>
+        <v>12.939243461538458</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" s="1">
-        <v>2015</v>
+        <v>2014</v>
       </c>
       <c r="B26" s="4">
-        <v>16.879134133333327</v>
+        <v>16.304540920716121</v>
       </c>
       <c r="C26" s="2">
-        <v>12.659690234374999</v>
+        <v>11.953458687258692</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" s="1">
-        <v>2016</v>
+        <v>2015</v>
       </c>
       <c r="B27" s="4">
-        <v>17.274034540389984</v>
+        <v>16.879134133333327</v>
       </c>
       <c r="C27" s="2">
-        <v>13.551704705882358</v>
+        <v>12.659690234374999</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
-        <v>2017</v>
+        <v>2016</v>
       </c>
       <c r="B28" s="4">
-        <v>18.29688942307693</v>
+        <v>17.274034540389984</v>
       </c>
       <c r="C28" s="2">
-        <v>14.089071808510633</v>
+        <v>13.551704705882358</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
-        <v>2018</v>
+        <v>2017</v>
       </c>
       <c r="B29" s="4">
-        <v>14.272313725490198</v>
+        <v>18.29688942307693</v>
       </c>
       <c r="C29" s="2">
-        <v>12.7836328125</v>
+        <v>14.089071808510633</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
-        <v>2019</v>
-      </c>
-      <c r="B30" s="1">
-        <v>13.830384615384617</v>
-      </c>
-      <c r="C30" s="5">
-        <v>12.593730769230801</v>
+        <v>2018</v>
+      </c>
+      <c r="B30" s="4">
+        <v>14.272313725490198</v>
+      </c>
+      <c r="C30" s="2">
+        <v>12.7836328125</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
-        <v>2020</v>
-      </c>
-      <c r="B31">
-        <v>16.89941520467837</v>
-      </c>
-      <c r="C31">
-        <v>15.350872093023261</v>
+        <v>2019</v>
+      </c>
+      <c r="B31" s="1">
+        <v>13.830384615384617</v>
+      </c>
+      <c r="C31" s="5">
+        <v>12.593730769230801</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" s="1">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="B32">
-        <v>16.655342465753421</v>
+        <v>16.89941520467837</v>
       </c>
       <c r="C32">
-        <v>15.067545454545453</v>
+        <v>15.350872093023261</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" s="1">
+        <v>2021</v>
+      </c>
+      <c r="B33">
+        <v>16.655342465753421</v>
+      </c>
+      <c r="C33">
+        <v>15.067545454545453</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" s="1">
         <v>2022</v>
       </c>
-      <c r="B33" s="1">
+      <c r="B34" s="1">
         <v>14.861021276595743</v>
       </c>
-      <c r="C33" s="2">
+      <c r="C34" s="2">
         <v>13.865529953917058</v>
       </c>
     </row>
-    <row r="34" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="1">
+    <row r="35" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A35" s="1">
         <v>2023</v>
       </c>
-      <c r="B34" s="6">
+      <c r="B35" s="6">
         <v>15.738356164383561</v>
       </c>
-      <c r="C34" s="6">
+      <c r="C35" s="6">
         <v>14.32657534246575</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A35" s="7">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36" s="7">
         <v>2024</v>
       </c>
-      <c r="B35" s="8">
+      <c r="B36" s="8">
         <v>15.097523809523805</v>
       </c>
-      <c r="C35" s="9">
+      <c r="C36" s="9">
         <v>13.372009569377994</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A36" s="46">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37" s="46">
         <v>2025</v>
       </c>
-      <c r="B36" s="8">
+      <c r="B37" s="8">
         <v>14.68</v>
       </c>
-      <c r="C36" s="9">
+      <c r="C37" s="9">
         <v>12.8</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A37" s="8"/>
-      <c r="B37" s="8"/>
-      <c r="C37" s="9"/>
-    </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A38" s="10"/>
+      <c r="A38" s="8">
+        <v>2026</v>
+      </c>
+      <c r="B38" s="8"/>
+      <c r="C38" s="9"/>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A39" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>